<commit_message>
Validated description, cited guidance, message
</commit_message>
<xml_diff>
--- a/rules/CORE-000251/negative/01/data/unit-test-coreid-CG0067-negative.xlsx
+++ b/rules/CORE-000251/negative/01/data/unit-test-coreid-CG0067-negative.xlsx
@@ -509,7 +509,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F2"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="str">
@@ -545,35 +545,15 @@
         <v>6</v>
       </c>
       <c r="E2" s="4" t="str">
-        <v>$ds_dsdecod</v>
+        <v>SSSTRESC</v>
       </c>
       <c r="F2" s="4" t="str">
-        <v>[ABSENT]</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="4">
-        <v>1</v>
-      </c>
-      <c r="B3" s="4" t="str">
-        <v>ss.xpt</v>
-      </c>
-      <c r="C3" s="4" t="str">
-        <v>Record</v>
-      </c>
-      <c r="D3" s="4">
-        <v>6</v>
-      </c>
-      <c r="E3" s="4" t="str">
-        <v>SSSTRESC</v>
-      </c>
-      <c r="F3" s="4" t="str">
         <v>DEAD</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F2"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>